<commit_message>
Updated estimate for home charging power
</commit_message>
<xml_diff>
--- a/InputData/trans/AVCC/Avg Vehicle Charger Capacity.xlsx
+++ b/InputData/trans/AVCC/Avg Vehicle Charger Capacity.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\trans\AVCC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\trans\AVCC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F441F22C-13F1-4168-BD58-8232EDA356FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31C09505-F5DC-4495-A821-AAF9FC0450FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{661390DE-D06E-402F-B49F-05F85B2DF025}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="11370" xr2:uid="{661390DE-D06E-402F-B49F-05F85B2DF025}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="9" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="28">
   <si>
     <t>ships</t>
   </si>
@@ -94,16 +94,39 @@
   </si>
   <si>
     <t>Average charger capacity (kW)</t>
+  </si>
+  <si>
+    <t>L1 vs L2 home charging split</t>
+  </si>
+  <si>
+    <t>JDPower</t>
+  </si>
+  <si>
+    <t>Home Charging Satisfaction a Bright Spot among Electric Vehicle Owners, JD Power Finds</t>
+  </si>
+  <si>
+    <t>https://www.jdpower.com/business/press-releases/2024-us-electric-vehicle-experience-evx-home-charging-study?utm_source=chatgpt.com</t>
+  </si>
+  <si>
+    <t>JDPower finds 84% of EV owners who charge at home use L2 permanently mounted charging stations.</t>
+  </si>
+  <si>
+    <t>L1 charging is roughly 1.4 kW.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L2 charging depends on setup, but 7.2 kW (30 A) is standard; some setups like Tesla wall chargers are </t>
+  </si>
+  <si>
+    <t xml:space="preserve">10-11 kW. So we use 8.5 kW as an approximate value given we lack better data. </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="###0.00_)"/>
-    <numFmt numFmtId="167" formatCode="0.0"/>
-    <numFmt numFmtId="169" formatCode="#,##0_)"/>
+    <numFmt numFmtId="166" formatCode="#,##0_)"/>
   </numFmts>
   <fonts count="31" x14ac:knownFonts="1">
     <font>
@@ -802,7 +825,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="8">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="29" fillId="0" borderId="8">
+    <xf numFmtId="166" fontId="29" fillId="0" borderId="8">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0"/>
@@ -823,12 +846,12 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="62">
     <cellStyle name="20% - Accent1" xfId="34" builtinId="30" customBuiltin="1"/>
@@ -1229,7 +1252,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="132.26953125" customWidth="1"/>
@@ -1299,13 +1322,76 @@
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A16" s="1" t="s">
+      <c r="B16" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B17" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B18" s="8">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B19" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B20" s="7" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B21" s="7"/>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
         <v>18</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A26" s="11">
+        <v>0.84</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A29">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A33">
+        <v>8.5</v>
       </c>
     </row>
   </sheetData>
@@ -1342,24 +1428,25 @@
       <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="10">
-        <v>7.5</v>
-      </c>
-      <c r="C2" s="11">
-        <f>B2</f>
-        <v>7.5</v>
+      <c r="B2" s="12">
+        <f>About!A33*About!A26+About!A29*(1-About!A26)</f>
+        <v>7.3639999999999999</v>
+      </c>
+      <c r="C2" s="12">
+        <f t="shared" ref="C2:C7" si="0">B2</f>
+        <v>7.3639999999999999</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="12">
+      <c r="B3" s="10">
         <f>(100-22)/2+22</f>
         <v>61</v>
       </c>
-      <c r="C3" s="12">
-        <f>B3</f>
+      <c r="C3" s="10">
+        <f t="shared" si="0"/>
         <v>61</v>
       </c>
     </row>
@@ -1367,11 +1454,11 @@
       <c r="A4" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="12">
+      <c r="B4" s="10">
         <v>0</v>
       </c>
-      <c r="C4" s="12">
-        <f>B4</f>
+      <c r="C4" s="10">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -1383,7 +1470,7 @@
         <v>0</v>
       </c>
       <c r="C5">
-        <f>B5</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -1395,7 +1482,7 @@
         <v>0</v>
       </c>
       <c r="C6">
-        <f>B6</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -1403,13 +1490,13 @@
       <c r="A7" t="s">
         <v>6</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="12">
         <f>B2</f>
-        <v>7.5</v>
-      </c>
-      <c r="C7">
-        <f>B7</f>
-        <v>7.5</v>
+        <v>7.3639999999999999</v>
+      </c>
+      <c r="C7" s="12">
+        <f t="shared" si="0"/>
+        <v>7.3639999999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>